<commit_message>
added output file dvt_excel.xlsx
</commit_message>
<xml_diff>
--- a/dvt_excel.xlsx
+++ b/dvt_excel.xlsx
@@ -516,7 +516,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:43</t>
+          <t>2026-03-11 15:04:50</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -526,7 +526,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Reg 0x00: OUT=0x0001, CE=0, STATUS=0 (OK)</t>
+          <t>Reg 0x00: OUT=0x8000, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:43</t>
+          <t>2026-03-11 15:04:50</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:43</t>
+          <t>2026-03-11 15:04:50</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:43</t>
+          <t>2026-03-11 15:04:50</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:43</t>
+          <t>2026-03-11 15:04:51</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:43</t>
+          <t>2026-03-11 15:04:51</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:43</t>
+          <t>2026-03-11 15:04:51</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:44</t>
+          <t>2026-03-11 15:04:51</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:44</t>
+          <t>2026-03-11 15:04:51</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:44</t>
+          <t>2026-03-11 15:04:51</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:44</t>
+          <t>2026-03-11 15:04:51</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:44</t>
+          <t>2026-03-11 15:04:51</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1092,7 +1092,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:44</t>
+          <t>2026-03-11 15:04:51</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:44</t>
+          <t>2026-03-11 15:04:51</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:44</t>
+          <t>2026-03-11 15:04:51</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1236,7 +1236,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:44</t>
+          <t>2026-03-11 15:04:52</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:44</t>
+          <t>2026-03-11 15:04:52</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:45</t>
+          <t>2026-03-11 15:04:52</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1380,7 +1380,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:45</t>
+          <t>2026-03-11 15:04:52</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1428,7 +1428,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:45</t>
+          <t>2026-03-11 15:04:52</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:45</t>
+          <t>2026-03-11 15:04:52</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:45</t>
+          <t>2026-03-11 15:04:52</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:45</t>
+          <t>2026-03-11 15:04:52</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:45</t>
+          <t>2026-03-11 15:04:52</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:45</t>
+          <t>2026-03-11 15:04:52</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:45</t>
+          <t>2026-03-11 15:04:52</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:45</t>
+          <t>2026-03-11 15:04:53</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:45</t>
+          <t>2026-03-11 15:04:53</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:46</t>
+          <t>2026-03-11 15:04:53</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:46</t>
+          <t>2026-03-11 15:04:53</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:46</t>
+          <t>2026-03-11 15:04:53</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2004,7 +2004,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:46</t>
+          <t>2026-03-11 15:04:53</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2052,7 +2052,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:46</t>
+          <t>2026-03-11 15:04:53</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2062,7 +2062,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Reg 0x20: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
+          <t>Reg 0x20: OUT=0xD080, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -2100,7 +2100,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:46</t>
+          <t>2026-03-11 15:04:53</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2110,7 +2110,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Reg 0x21: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
+          <t>Reg 0x21: OUT=0xD585, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -2148,7 +2148,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:46</t>
+          <t>2026-03-11 15:04:53</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:46</t>
+          <t>2026-03-11 15:04:53</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:46</t>
+          <t>2026-03-11 15:04:54</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2292,7 +2292,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:46</t>
+          <t>2026-03-11 15:04:54</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:46</t>
+          <t>2026-03-11 15:04:54</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2388,7 +2388,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:47</t>
+          <t>2026-03-11 15:04:54</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2436,7 +2436,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:47</t>
+          <t>2026-03-11 15:04:54</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Reg 0x28: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
+          <t>Reg 0x28: OUT=0x1FBF, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -2484,7 +2484,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:47</t>
+          <t>2026-03-11 15:04:54</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2494,7 +2494,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Reg 0x29: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
+          <t>Reg 0x29: OUT=0x000F, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -2532,7 +2532,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:47</t>
+          <t>2026-03-11 15:04:54</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2542,7 +2542,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Reg 0x2A: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
+          <t>Reg 0x2A: OUT=0x0D0D, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:47</t>
+          <t>2026-03-11 15:04:54</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2628,7 +2628,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:47</t>
+          <t>2026-03-11 15:04:54</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:47</t>
+          <t>2026-03-11 15:04:54</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2724,7 +2724,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:47</t>
+          <t>2026-03-11 15:04:54</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:47</t>
+          <t>2026-03-11 15:04:55</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2820,7 +2820,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:47</t>
+          <t>2026-03-11 15:04:55</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:47</t>
+          <t>2026-03-11 15:04:55</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -2916,7 +2916,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:48</t>
+          <t>2026-03-11 15:04:55</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -2964,7 +2964,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:48</t>
+          <t>2026-03-11 15:04:55</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2974,7 +2974,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Reg 0x33: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
+          <t>Reg 0x33: OUT=0x0002, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -3012,7 +3012,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:48</t>
+          <t>2026-03-11 15:04:55</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3060,7 +3060,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:48</t>
+          <t>2026-03-11 15:04:55</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:48</t>
+          <t>2026-03-11 15:04:55</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3156,7 +3156,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:48</t>
+          <t>2026-03-11 15:04:55</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3204,7 +3204,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:48</t>
+          <t>2026-03-11 15:04:55</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -3252,7 +3252,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:48</t>
+          <t>2026-03-11 15:04:55</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -3300,7 +3300,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:48</t>
+          <t>2026-03-11 15:04:56</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3348,7 +3348,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:48</t>
+          <t>2026-03-11 15:04:56</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3396,7 +3396,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:49</t>
+          <t>2026-03-11 15:04:56</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3444,7 +3444,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:49</t>
+          <t>2026-03-11 15:04:56</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3492,7 +3492,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:49</t>
+          <t>2026-03-11 15:04:56</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3540,7 +3540,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:49</t>
+          <t>2026-03-11 15:04:56</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3588,7 +3588,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:49</t>
+          <t>2026-03-11 15:04:56</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3636,7 +3636,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:49</t>
+          <t>2026-03-11 15:04:56</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3684,7 +3684,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:49</t>
+          <t>2026-03-11 15:04:56</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -3732,7 +3732,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:49</t>
+          <t>2026-03-11 15:04:56</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3780,7 +3780,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:49</t>
+          <t>2026-03-11 15:04:57</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3828,7 +3828,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:49</t>
+          <t>2026-03-11 15:04:57</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -3876,7 +3876,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:49</t>
+          <t>2026-03-11 15:04:57</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -3924,7 +3924,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:50</t>
+          <t>2026-03-11 15:04:57</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -3972,7 +3972,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:50</t>
+          <t>2026-03-11 15:04:57</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -4020,7 +4020,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:50</t>
+          <t>2026-03-11 15:04:57</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -4068,7 +4068,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:50</t>
+          <t>2026-03-11 15:04:57</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -4116,7 +4116,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:50</t>
+          <t>2026-03-11 15:04:57</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:50</t>
+          <t>2026-03-11 15:04:57</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -4212,7 +4212,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:50</t>
+          <t>2026-03-11 15:04:57</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -4260,7 +4260,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:50</t>
+          <t>2026-03-11 15:04:57</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -4308,7 +4308,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:50</t>
+          <t>2026-03-11 15:04:58</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -4356,7 +4356,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:50</t>
+          <t>2026-03-11 15:04:58</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -4404,7 +4404,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:50</t>
+          <t>2026-03-11 15:04:58</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -4452,7 +4452,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:51</t>
+          <t>2026-03-11 15:04:58</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -4500,7 +4500,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:51</t>
+          <t>2026-03-11 15:04:58</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -4548,7 +4548,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:51</t>
+          <t>2026-03-11 15:04:58</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -4596,7 +4596,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:51</t>
+          <t>2026-03-11 15:04:58</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -4644,7 +4644,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:51</t>
+          <t>2026-03-11 15:04:58</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -4673,16 +4673,16 @@
         <v>0</v>
       </c>
       <c r="D89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -4692,7 +4692,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:51</t>
+          <t>2026-03-11 15:04:58</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -4702,7 +4702,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>Reg 0x57: OUT=0x0000, CE=0, STATUS=1 (XE)</t>
+          <t>Reg 0x57: OUT=0x0008, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -4721,16 +4721,16 @@
         <v>0</v>
       </c>
       <c r="D90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -4740,7 +4740,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:51</t>
+          <t>2026-03-11 15:04:58</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -4750,7 +4750,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>Reg 0x58: OUT=0x0000, CE=0, STATUS=1 (XE)</t>
+          <t>Reg 0x58: OUT=0x0004, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -4769,16 +4769,16 @@
         <v>0</v>
       </c>
       <c r="D91" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -4788,7 +4788,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:51</t>
+          <t>2026-03-11 15:04:58</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -4798,7 +4798,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>Reg 0x59: OUT=0x0000, CE=0, STATUS=1 (XE)</t>
+          <t>Reg 0x59: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -4817,16 +4817,16 @@
         <v>0</v>
       </c>
       <c r="D92" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -4836,7 +4836,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:51</t>
+          <t>2026-03-11 15:04:59</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -4846,7 +4846,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>Reg 0x5A: OUT=0x0000, CE=0, STATUS=1 (XE)</t>
+          <t>Reg 0x5A: OUT=0x0064, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -4865,16 +4865,16 @@
         <v>0</v>
       </c>
       <c r="D93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -4884,7 +4884,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:51</t>
+          <t>2026-03-11 15:04:59</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -4894,7 +4894,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>Reg 0x5B: OUT=0x0000, CE=0, STATUS=1 (XE)</t>
+          <t>Reg 0x5B: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -4913,16 +4913,16 @@
         <v>0</v>
       </c>
       <c r="D94" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -4932,7 +4932,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:52</t>
+          <t>2026-03-11 15:04:59</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -4942,7 +4942,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>Reg 0x5C: OUT=0x0000, CE=0, STATUS=1 (XE)</t>
+          <t>Reg 0x5C: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -4961,16 +4961,16 @@
         <v>0</v>
       </c>
       <c r="D95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -4980,7 +4980,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:52</t>
+          <t>2026-03-11 15:04:59</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -4990,7 +4990,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>Reg 0x5D: OUT=0x0000, CE=0, STATUS=1 (XE)</t>
+          <t>Reg 0x5D: OUT=0xFE0C, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -5009,16 +5009,16 @@
         <v>0</v>
       </c>
       <c r="D96" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -5028,7 +5028,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:52</t>
+          <t>2026-03-11 15:04:59</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -5038,7 +5038,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>Reg 0x5E: OUT=0x0000, CE=0, STATUS=1 (XE)</t>
+          <t>Reg 0x5E: OUT=0x1B58, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -5057,16 +5057,16 @@
         <v>0</v>
       </c>
       <c r="D97" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -5076,7 +5076,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:52</t>
+          <t>2026-03-11 15:04:59</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -5086,7 +5086,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>Reg 0x5F: OUT=0x0000, CE=0, STATUS=1 (XE)</t>
+          <t>Reg 0x5F: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -5105,16 +5105,16 @@
         <v>0</v>
       </c>
       <c r="D98" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -5124,7 +5124,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:52</t>
+          <t>2026-03-11 15:04:59</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>Reg 0x60: OUT=0x0000, CE=0, STATUS=1 (XE)</t>
+          <t>Reg 0x60: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -5153,16 +5153,16 @@
         <v>0</v>
       </c>
       <c r="D99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -5172,7 +5172,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:52</t>
+          <t>2026-03-11 15:04:59</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -5182,7 +5182,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>Reg 0x61: OUT=0x0000, CE=0, STATUS=1 (XE)</t>
+          <t>Reg 0x61: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:52</t>
+          <t>2026-03-11 15:04:59</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -5249,16 +5249,16 @@
         <v>0</v>
       </c>
       <c r="D101" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -5268,7 +5268,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:52</t>
+          <t>2026-03-11 15:04:59</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -5278,7 +5278,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>Reg 0x63: OUT=0x0000, CE=0, STATUS=1 (XE)</t>
+          <t>Reg 0x63: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -5297,16 +5297,16 @@
         <v>0</v>
       </c>
       <c r="D102" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -5316,7 +5316,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:52</t>
+          <t>2026-03-11 15:05:00</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -5326,7 +5326,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>Reg 0x64: OUT=0x0000, CE=0, STATUS=1 (XE)</t>
+          <t>Reg 0x64: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:52</t>
+          <t>2026-03-11 15:05:00</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -5412,7 +5412,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:52</t>
+          <t>2026-03-11 15:05:00</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -5460,7 +5460,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:53</t>
+          <t>2026-03-11 15:05:00</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -5508,7 +5508,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:53</t>
+          <t>2026-03-11 15:05:00</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -5537,16 +5537,16 @@
         <v>0</v>
       </c>
       <c r="D107" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -5556,7 +5556,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:53</t>
+          <t>2026-03-11 15:05:00</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -5566,7 +5566,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>Reg 0x69: OUT=0x0000, CE=0, STATUS=1 (XE)</t>
+          <t>Reg 0x69: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -5585,16 +5585,16 @@
         <v>0</v>
       </c>
       <c r="D108" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -5604,7 +5604,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:53</t>
+          <t>2026-03-11 15:05:00</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>Reg 0x6A: OUT=0x0000, CE=0, STATUS=1 (XE)</t>
+          <t>Reg 0x6A: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -5633,16 +5633,16 @@
         <v>0</v>
       </c>
       <c r="D109" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -5652,7 +5652,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:53</t>
+          <t>2026-03-11 15:05:00</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -5662,7 +5662,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>Reg 0x6B: OUT=0x0000, CE=0, STATUS=1 (XE)</t>
+          <t>Reg 0x6B: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -5700,7 +5700,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:53</t>
+          <t>2026-03-11 15:05:00</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -5748,7 +5748,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:53</t>
+          <t>2026-03-11 15:05:00</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -5796,7 +5796,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:53</t>
+          <t>2026-03-11 15:05:00</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -5844,7 +5844,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:53</t>
+          <t>2026-03-11 15:05:01</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -5892,7 +5892,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:53</t>
+          <t>2026-03-11 15:05:01</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -5940,7 +5940,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:54</t>
+          <t>2026-03-11 15:05:01</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -5988,7 +5988,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:54</t>
+          <t>2026-03-11 15:05:01</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -6036,7 +6036,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:54</t>
+          <t>2026-03-11 15:05:01</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -6084,7 +6084,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:54</t>
+          <t>2026-03-11 15:05:01</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -6132,7 +6132,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:54</t>
+          <t>2026-03-11 15:05:01</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -6180,7 +6180,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:54</t>
+          <t>2026-03-11 15:05:01</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -6228,7 +6228,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:54</t>
+          <t>2026-03-11 15:05:01</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -6276,7 +6276,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:54</t>
+          <t>2026-03-11 15:05:01</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -6324,7 +6324,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:54</t>
+          <t>2026-03-11 15:05:01</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -6372,7 +6372,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:54</t>
+          <t>2026-03-11 15:05:02</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -6420,7 +6420,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:54</t>
+          <t>2026-03-11 15:05:02</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -6468,7 +6468,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:55</t>
+          <t>2026-03-11 15:05:02</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -6516,7 +6516,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:55</t>
+          <t>2026-03-11 15:05:02</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:55</t>
+          <t>2026-03-11 15:05:02</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -6612,7 +6612,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:55</t>
+          <t>2026-03-11 15:05:02</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -6660,7 +6660,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:55</t>
+          <t>2026-03-11 15:05:02</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -6708,7 +6708,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:55</t>
+          <t>2026-03-11 15:05:02</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -6756,7 +6756,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:55</t>
+          <t>2026-03-11 15:05:02</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -6804,7 +6804,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:55</t>
+          <t>2026-03-11 15:05:02</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -6852,7 +6852,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:55</t>
+          <t>2026-03-11 15:05:03</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -6900,7 +6900,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:55</t>
+          <t>2026-03-11 15:05:03</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -6948,7 +6948,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:56</t>
+          <t>2026-03-11 15:05:03</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -6996,7 +6996,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:56</t>
+          <t>2026-03-11 15:05:03</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -7044,7 +7044,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:56</t>
+          <t>2026-03-11 15:05:03</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -7092,7 +7092,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:56</t>
+          <t>2026-03-11 15:05:03</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -7102,7 +7102,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>Reg 0x89: OUT=0x000A, CE=0, STATUS=0 (OK)</t>
+          <t>Reg 0x89: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -7140,7 +7140,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:56</t>
+          <t>2026-03-11 15:05:03</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -7150,7 +7150,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>Reg 0x8A: OUT=0x0014, CE=0, STATUS=0 (OK)</t>
+          <t>Reg 0x8A: OUT=0x000A, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -7188,7 +7188,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:56</t>
+          <t>2026-03-11 15:05:03</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -7198,7 +7198,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>Reg 0x8B: OUT=0x001E, CE=0, STATUS=0 (OK)</t>
+          <t>Reg 0x8B: OUT=0x000A, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -7236,7 +7236,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:56</t>
+          <t>2026-03-11 15:05:03</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -7284,7 +7284,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:56</t>
+          <t>2026-03-11 15:05:03</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -7332,7 +7332,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:56</t>
+          <t>2026-03-11 15:05:03</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -7380,7 +7380,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:56</t>
+          <t>2026-03-11 15:05:04</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -7428,7 +7428,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:56</t>
+          <t>2026-03-11 15:05:04</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -7476,7 +7476,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:57</t>
+          <t>2026-03-11 15:05:04</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -7505,16 +7505,16 @@
         <v>0</v>
       </c>
       <c r="D148" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>XE</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -7524,7 +7524,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:57</t>
+          <t>2026-03-11 15:05:04</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -7534,7 +7534,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>Reg 0x92: OUT=0x0000, CE=0, STATUS=1 (XE)</t>
+          <t>Reg 0x92: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -7572,7 +7572,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:57</t>
+          <t>2026-03-11 15:05:04</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -7620,7 +7620,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:57</t>
+          <t>2026-03-11 15:05:04</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -7668,7 +7668,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:57</t>
+          <t>2026-03-11 15:05:04</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -7716,7 +7716,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:57</t>
+          <t>2026-03-11 15:05:04</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:57</t>
+          <t>2026-03-11 15:05:04</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -7812,7 +7812,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:57</t>
+          <t>2026-03-11 15:05:04</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -7860,7 +7860,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:57</t>
+          <t>2026-03-11 15:05:04</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -7908,7 +7908,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:57</t>
+          <t>2026-03-11 15:05:05</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -7956,7 +7956,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:57</t>
+          <t>2026-03-11 15:05:05</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -8004,7 +8004,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:58</t>
+          <t>2026-03-11 15:05:05</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -8052,7 +8052,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:58</t>
+          <t>2026-03-11 15:05:05</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -8100,7 +8100,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:58</t>
+          <t>2026-03-11 15:05:05</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -8148,7 +8148,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:58</t>
+          <t>2026-03-11 15:05:05</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -8196,7 +8196,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:58</t>
+          <t>2026-03-11 15:05:05</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -8244,7 +8244,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:58</t>
+          <t>2026-03-11 15:05:05</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -8292,7 +8292,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:58</t>
+          <t>2026-03-11 15:05:05</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -8340,7 +8340,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:58</t>
+          <t>2026-03-11 15:05:05</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -8388,7 +8388,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:58</t>
+          <t>2026-03-11 15:05:06</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -8436,7 +8436,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:58</t>
+          <t>2026-03-11 15:05:06</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -8484,7 +8484,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:59</t>
+          <t>2026-03-11 15:05:06</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -8532,7 +8532,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:59</t>
+          <t>2026-03-11 15:05:06</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -8580,7 +8580,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:59</t>
+          <t>2026-03-11 15:05:06</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -8628,7 +8628,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:59</t>
+          <t>2026-03-11 15:05:06</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -8676,7 +8676,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:59</t>
+          <t>2026-03-11 15:05:06</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -8724,7 +8724,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:59</t>
+          <t>2026-03-11 15:05:06</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:59</t>
+          <t>2026-03-11 15:05:06</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -8820,7 +8820,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:59</t>
+          <t>2026-03-11 15:05:06</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -8868,7 +8868,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:59</t>
+          <t>2026-03-11 15:05:06</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -8916,7 +8916,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:59</t>
+          <t>2026-03-11 15:05:07</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>2026-03-11 11:39:59</t>
+          <t>2026-03-11 15:05:07</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -9012,7 +9012,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:00</t>
+          <t>2026-03-11 15:05:07</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -9060,7 +9060,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:00</t>
+          <t>2026-03-11 15:05:07</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -9108,7 +9108,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:00</t>
+          <t>2026-03-11 15:05:07</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -9156,7 +9156,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:00</t>
+          <t>2026-03-11 15:05:07</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -9204,7 +9204,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:00</t>
+          <t>2026-03-11 15:05:07</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -9252,7 +9252,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:00</t>
+          <t>2026-03-11 15:05:07</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -9300,7 +9300,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:00</t>
+          <t>2026-03-11 15:05:07</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -9348,7 +9348,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:00</t>
+          <t>2026-03-11 15:05:07</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -9396,7 +9396,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:00</t>
+          <t>2026-03-11 15:05:08</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -9444,7 +9444,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:00</t>
+          <t>2026-03-11 15:05:08</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -9492,7 +9492,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:00</t>
+          <t>2026-03-11 15:05:08</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -9540,7 +9540,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:01</t>
+          <t>2026-03-11 15:05:08</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -9588,7 +9588,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:01</t>
+          <t>2026-03-11 15:05:08</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -9636,7 +9636,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:01</t>
+          <t>2026-03-11 15:05:08</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -9684,7 +9684,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:01</t>
+          <t>2026-03-11 15:05:08</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -9732,7 +9732,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:01</t>
+          <t>2026-03-11 15:05:08</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -9780,7 +9780,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:01</t>
+          <t>2026-03-11 15:05:08</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -9828,7 +9828,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:01</t>
+          <t>2026-03-11 15:05:08</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -9876,7 +9876,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:01</t>
+          <t>2026-03-11 15:05:08</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -9924,7 +9924,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:01</t>
+          <t>2026-03-11 15:05:09</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -9972,7 +9972,7 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:01</t>
+          <t>2026-03-11 15:05:09</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -10020,7 +10020,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:02</t>
+          <t>2026-03-11 15:05:09</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -10068,7 +10068,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:02</t>
+          <t>2026-03-11 15:05:09</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -10116,7 +10116,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:02</t>
+          <t>2026-03-11 15:05:09</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:02</t>
+          <t>2026-03-11 15:05:09</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -10212,7 +10212,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:02</t>
+          <t>2026-03-11 15:05:09</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -10260,7 +10260,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:02</t>
+          <t>2026-03-11 15:05:09</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -10308,7 +10308,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:02</t>
+          <t>2026-03-11 15:05:09</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -10356,7 +10356,7 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:02</t>
+          <t>2026-03-11 15:05:09</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -10404,7 +10404,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:02</t>
+          <t>2026-03-11 15:05:09</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -10452,7 +10452,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:02</t>
+          <t>2026-03-11 15:05:10</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
@@ -10500,7 +10500,7 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:02</t>
+          <t>2026-03-11 15:05:10</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
@@ -10548,7 +10548,7 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:03</t>
+          <t>2026-03-11 15:05:10</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
@@ -10596,7 +10596,7 @@
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:03</t>
+          <t>2026-03-11 15:05:10</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
@@ -10644,7 +10644,7 @@
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:03</t>
+          <t>2026-03-11 15:05:10</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
@@ -10692,7 +10692,7 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:03</t>
+          <t>2026-03-11 15:05:10</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
@@ -10740,7 +10740,7 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:03</t>
+          <t>2026-03-11 15:05:10</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
@@ -10788,7 +10788,7 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:03</t>
+          <t>2026-03-11 15:05:10</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
@@ -10836,7 +10836,7 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:03</t>
+          <t>2026-03-11 15:05:10</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
@@ -10884,7 +10884,7 @@
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:03</t>
+          <t>2026-03-11 15:05:10</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
@@ -10932,7 +10932,7 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:03</t>
+          <t>2026-03-11 15:05:10</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
@@ -10980,7 +10980,7 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:03</t>
+          <t>2026-03-11 15:05:11</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
@@ -11028,7 +11028,7 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:04</t>
+          <t>2026-03-11 15:05:11</t>
         </is>
       </c>
       <c r="I221" t="inlineStr">
@@ -11076,7 +11076,7 @@
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:04</t>
+          <t>2026-03-11 15:05:11</t>
         </is>
       </c>
       <c r="I222" t="inlineStr">
@@ -11124,7 +11124,7 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:04</t>
+          <t>2026-03-11 15:05:11</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
@@ -11172,7 +11172,7 @@
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:04</t>
+          <t>2026-03-11 15:05:11</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
@@ -11220,7 +11220,7 @@
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:04</t>
+          <t>2026-03-11 15:05:11</t>
         </is>
       </c>
       <c r="I225" t="inlineStr">
@@ -11268,7 +11268,7 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:04</t>
+          <t>2026-03-11 15:05:11</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
@@ -11316,7 +11316,7 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:04</t>
+          <t>2026-03-11 15:05:11</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
@@ -11364,7 +11364,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:04</t>
+          <t>2026-03-11 15:05:11</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
@@ -11412,7 +11412,7 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:04</t>
+          <t>2026-03-11 15:05:11</t>
         </is>
       </c>
       <c r="I229" t="inlineStr">
@@ -11460,7 +11460,7 @@
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:04</t>
+          <t>2026-03-11 15:05:12</t>
         </is>
       </c>
       <c r="I230" t="inlineStr">
@@ -11508,7 +11508,7 @@
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:04</t>
+          <t>2026-03-11 15:05:12</t>
         </is>
       </c>
       <c r="I231" t="inlineStr">
@@ -11556,7 +11556,7 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:05</t>
+          <t>2026-03-11 15:05:12</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
@@ -11604,7 +11604,7 @@
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:05</t>
+          <t>2026-03-11 15:05:12</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
@@ -11652,7 +11652,7 @@
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:05</t>
+          <t>2026-03-11 15:05:12</t>
         </is>
       </c>
       <c r="I234" t="inlineStr">
@@ -11700,7 +11700,7 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:05</t>
+          <t>2026-03-11 15:05:12</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
@@ -11748,7 +11748,7 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:05</t>
+          <t>2026-03-11 15:05:12</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
@@ -11796,7 +11796,7 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:05</t>
+          <t>2026-03-11 15:05:12</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
@@ -11844,7 +11844,7 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:05</t>
+          <t>2026-03-11 15:05:12</t>
         </is>
       </c>
       <c r="I238" t="inlineStr">
@@ -11892,7 +11892,7 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:05</t>
+          <t>2026-03-11 15:05:12</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
@@ -11940,7 +11940,7 @@
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:05</t>
+          <t>2026-03-11 15:05:12</t>
         </is>
       </c>
       <c r="I240" t="inlineStr">
@@ -11988,7 +11988,7 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:05</t>
+          <t>2026-03-11 15:05:13</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
@@ -12036,7 +12036,7 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:05</t>
+          <t>2026-03-11 15:05:13</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
@@ -12084,7 +12084,7 @@
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:06</t>
+          <t>2026-03-11 15:05:13</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
@@ -12132,7 +12132,7 @@
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:06</t>
+          <t>2026-03-11 15:05:13</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">
@@ -12180,7 +12180,7 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:06</t>
+          <t>2026-03-11 15:05:13</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
@@ -12228,7 +12228,7 @@
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:06</t>
+          <t>2026-03-11 15:05:13</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
@@ -12276,7 +12276,7 @@
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:06</t>
+          <t>2026-03-11 15:05:13</t>
         </is>
       </c>
       <c r="I247" t="inlineStr">
@@ -12324,7 +12324,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:06</t>
+          <t>2026-03-11 15:05:13</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
@@ -12372,7 +12372,7 @@
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:06</t>
+          <t>2026-03-11 15:05:13</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
@@ -12420,7 +12420,7 @@
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:06</t>
+          <t>2026-03-11 15:05:14</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
@@ -12468,7 +12468,7 @@
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:06</t>
+          <t>2026-03-11 15:05:14</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
@@ -12516,7 +12516,7 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:06</t>
+          <t>2026-03-11 15:05:14</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
@@ -12564,7 +12564,7 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:07</t>
+          <t>2026-03-11 15:05:14</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
@@ -12612,7 +12612,7 @@
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:07</t>
+          <t>2026-03-11 15:05:14</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
@@ -12660,7 +12660,7 @@
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:07</t>
+          <t>2026-03-11 15:05:14</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
@@ -12708,7 +12708,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:07</t>
+          <t>2026-03-11 15:05:14</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -12756,7 +12756,7 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>2026-03-11 11:40:07</t>
+          <t>2026-03-11 15:05:14</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">

</xml_diff>

<commit_message>
Add dvt_excel.xlsx output file
</commit_message>
<xml_diff>
--- a/dvt_excel.xlsx
+++ b/dvt_excel.xlsx
@@ -577,7 +577,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:38</t>
+          <t>2026-03-11 17:37:20</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -651,7 +651,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:39</t>
+          <t>2026-03-11 17:37:21</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:40</t>
+          <t>2026-03-11 17:37:22</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:40</t>
+          <t>2026-03-11 17:37:22</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:41</t>
+          <t>2026-03-11 17:37:23</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:42</t>
+          <t>2026-03-11 17:37:24</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:42</t>
+          <t>2026-03-11 17:37:24</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:42</t>
+          <t>2026-03-11 17:37:24</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1206,7 +1206,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:43</t>
+          <t>2026-03-11 17:37:25</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:43</t>
+          <t>2026-03-11 17:37:25</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:43</t>
+          <t>2026-03-11 17:37:25</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:43</t>
+          <t>2026-03-11 17:37:25</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:43</t>
+          <t>2026-03-11 17:37:25</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:44</t>
+          <t>2026-03-11 17:37:26</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:44</t>
+          <t>2026-03-11 17:37:26</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:45</t>
+          <t>2026-03-11 17:37:27</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:45</t>
+          <t>2026-03-11 17:37:27</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1584,7 +1584,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:45</t>
+          <t>2026-03-11 17:37:27</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:46</t>
+          <t>2026-03-11 17:37:28</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:46</t>
+          <t>2026-03-11 17:37:28</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:46</t>
+          <t>2026-03-11 17:37:28</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:47</t>
+          <t>2026-03-11 17:37:29</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1871,7 +1871,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:47</t>
+          <t>2026-03-11 17:37:29</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:47</t>
+          <t>2026-03-11 17:37:29</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:47</t>
+          <t>2026-03-11 17:37:29</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:48</t>
+          <t>2026-03-11 17:37:30</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:48</t>
+          <t>2026-03-11 17:37:30</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -2136,7 +2136,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:48</t>
+          <t>2026-03-11 17:37:30</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:48</t>
+          <t>2026-03-11 17:37:30</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -2242,7 +2242,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:48</t>
+          <t>2026-03-11 17:37:30</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:48</t>
+          <t>2026-03-11 17:37:30</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:48</t>
+          <t>2026-03-11 17:37:30</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:48</t>
+          <t>2026-03-11 17:37:30</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -2454,7 +2454,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:48</t>
+          <t>2026-03-11 17:37:30</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:48</t>
+          <t>2026-03-11 17:37:30</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -2560,7 +2560,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:49</t>
+          <t>2026-03-11 17:37:30</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -2613,7 +2613,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:49</t>
+          <t>2026-03-11 17:37:31</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -2666,7 +2666,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:49</t>
+          <t>2026-03-11 17:37:31</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -2719,7 +2719,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:49</t>
+          <t>2026-03-11 17:37:31</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:49</t>
+          <t>2026-03-11 17:37:31</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2825,7 +2825,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:49</t>
+          <t>2026-03-11 17:37:31</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2878,7 +2878,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:49</t>
+          <t>2026-03-11 17:37:31</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:49</t>
+          <t>2026-03-11 17:37:31</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -2984,7 +2984,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:49</t>
+          <t>2026-03-11 17:37:31</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:49</t>
+          <t>2026-03-11 17:37:31</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -3090,7 +3090,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:49</t>
+          <t>2026-03-11 17:37:31</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:50</t>
+          <t>2026-03-11 17:37:32</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -3196,7 +3196,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:50</t>
+          <t>2026-03-11 17:37:32</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:50</t>
+          <t>2026-03-11 17:37:32</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -3302,7 +3302,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:50</t>
+          <t>2026-03-11 17:37:32</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:50</t>
+          <t>2026-03-11 17:37:32</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:50</t>
+          <t>2026-03-11 17:37:32</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -3461,7 +3461,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:50</t>
+          <t>2026-03-11 17:37:32</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:50</t>
+          <t>2026-03-11 17:37:32</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:50</t>
+          <t>2026-03-11 17:37:32</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -3620,7 +3620,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:50</t>
+          <t>2026-03-11 17:37:32</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -3673,7 +3673,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:50</t>
+          <t>2026-03-11 17:37:32</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -3726,7 +3726,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:51</t>
+          <t>2026-03-11 17:37:33</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:51</t>
+          <t>2026-03-11 17:37:33</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -3832,7 +3832,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:51</t>
+          <t>2026-03-11 17:37:33</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:51</t>
+          <t>2026-03-11 17:37:33</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -3938,7 +3938,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:51</t>
+          <t>2026-03-11 17:37:33</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -3991,7 +3991,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:51</t>
+          <t>2026-03-11 17:37:33</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -4044,7 +4044,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:51</t>
+          <t>2026-03-11 17:37:33</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -4097,7 +4097,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:51</t>
+          <t>2026-03-11 17:37:33</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -4150,7 +4150,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:51</t>
+          <t>2026-03-11 17:37:33</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4203,7 +4203,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:51</t>
+          <t>2026-03-11 17:37:33</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -4256,7 +4256,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:52</t>
+          <t>2026-03-11 17:37:33</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -4309,7 +4309,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:52</t>
+          <t>2026-03-11 17:37:34</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:52</t>
+          <t>2026-03-11 17:37:34</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -4415,7 +4415,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:52</t>
+          <t>2026-03-11 17:37:34</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -4468,7 +4468,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:52</t>
+          <t>2026-03-11 17:37:34</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -4521,7 +4521,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:52</t>
+          <t>2026-03-11 17:37:34</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -4574,7 +4574,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:52</t>
+          <t>2026-03-11 17:37:34</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:52</t>
+          <t>2026-03-11 17:37:34</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -4680,7 +4680,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:52</t>
+          <t>2026-03-11 17:37:34</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -4733,7 +4733,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:52</t>
+          <t>2026-03-11 17:37:34</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -4786,7 +4786,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:52</t>
+          <t>2026-03-11 17:37:34</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -4839,7 +4839,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:53</t>
+          <t>2026-03-11 17:37:35</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -4892,7 +4892,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:53</t>
+          <t>2026-03-11 17:37:35</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -4945,7 +4945,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:53</t>
+          <t>2026-03-11 17:37:35</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:53</t>
+          <t>2026-03-11 17:37:35</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -5051,7 +5051,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:53</t>
+          <t>2026-03-11 17:37:35</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -5104,7 +5104,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:53</t>
+          <t>2026-03-11 17:37:35</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:53</t>
+          <t>2026-03-11 17:37:35</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -5210,7 +5210,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:53</t>
+          <t>2026-03-11 17:37:35</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -5263,7 +5263,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:53</t>
+          <t>2026-03-11 17:37:35</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -5316,7 +5316,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:53</t>
+          <t>2026-03-11 17:37:35</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -5369,7 +5369,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:53</t>
+          <t>2026-03-11 17:37:35</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -5422,7 +5422,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:54</t>
+          <t>2026-03-11 17:37:36</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -5475,7 +5475,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:54</t>
+          <t>2026-03-11 17:37:36</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -5528,7 +5528,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:54</t>
+          <t>2026-03-11 17:37:36</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -5581,7 +5581,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:54</t>
+          <t>2026-03-11 17:37:36</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -5634,7 +5634,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:54</t>
+          <t>2026-03-11 17:37:36</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -5687,7 +5687,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:54</t>
+          <t>2026-03-11 17:37:36</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:54</t>
+          <t>2026-03-11 17:37:36</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -5793,7 +5793,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:54</t>
+          <t>2026-03-11 17:37:36</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -5846,7 +5846,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:54</t>
+          <t>2026-03-11 17:37:36</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -5899,7 +5899,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:54</t>
+          <t>2026-03-11 17:37:36</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -5952,7 +5952,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:54</t>
+          <t>2026-03-11 17:37:37</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -6005,7 +6005,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:55</t>
+          <t>2026-03-11 17:37:37</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -6058,7 +6058,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:55</t>
+          <t>2026-03-11 17:37:37</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:55</t>
+          <t>2026-03-11 17:37:37</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:55</t>
+          <t>2026-03-11 17:37:37</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -6217,7 +6217,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:55</t>
+          <t>2026-03-11 17:37:37</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -6270,7 +6270,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:55</t>
+          <t>2026-03-11 17:37:37</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:55</t>
+          <t>2026-03-11 17:37:37</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -6376,7 +6376,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:55</t>
+          <t>2026-03-11 17:37:37</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -6429,7 +6429,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:55</t>
+          <t>2026-03-11 17:37:37</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -6482,7 +6482,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:55</t>
+          <t>2026-03-11 17:37:37</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -6535,7 +6535,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:56</t>
+          <t>2026-03-11 17:37:38</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -6588,7 +6588,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:56</t>
+          <t>2026-03-11 17:37:38</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -6641,7 +6641,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:56</t>
+          <t>2026-03-11 17:37:38</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -6694,7 +6694,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:56</t>
+          <t>2026-03-11 17:37:38</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -6747,7 +6747,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:56</t>
+          <t>2026-03-11 17:37:38</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:56</t>
+          <t>2026-03-11 17:37:38</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -6853,7 +6853,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:56</t>
+          <t>2026-03-11 17:37:38</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -6906,7 +6906,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:56</t>
+          <t>2026-03-11 17:37:38</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -6959,7 +6959,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:56</t>
+          <t>2026-03-11 17:37:38</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -7012,7 +7012,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:56</t>
+          <t>2026-03-11 17:37:38</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -7065,7 +7065,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:57</t>
+          <t>2026-03-11 17:37:38</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -7118,7 +7118,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:57</t>
+          <t>2026-03-11 17:37:39</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -7171,7 +7171,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:57</t>
+          <t>2026-03-11 17:37:39</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -7224,7 +7224,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:57</t>
+          <t>2026-03-11 17:37:39</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -7277,7 +7277,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:57</t>
+          <t>2026-03-11 17:37:39</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -7330,7 +7330,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:57</t>
+          <t>2026-03-11 17:37:39</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -7383,7 +7383,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:57</t>
+          <t>2026-03-11 17:37:39</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
@@ -7436,7 +7436,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:57</t>
+          <t>2026-03-11 17:37:39</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -7489,7 +7489,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:57</t>
+          <t>2026-03-11 17:37:39</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
@@ -7542,7 +7542,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:57</t>
+          <t>2026-03-11 17:37:39</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
@@ -7595,7 +7595,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:57</t>
+          <t>2026-03-11 17:37:39</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -7648,7 +7648,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:58</t>
+          <t>2026-03-11 17:37:39</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -7701,7 +7701,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:58</t>
+          <t>2026-03-11 17:37:40</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -7754,7 +7754,7 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:58</t>
+          <t>2026-03-11 17:37:40</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
@@ -7807,7 +7807,7 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:58</t>
+          <t>2026-03-11 17:37:40</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
@@ -7860,7 +7860,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:58</t>
+          <t>2026-03-11 17:37:40</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
@@ -7913,7 +7913,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:58</t>
+          <t>2026-03-11 17:37:40</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
@@ -7966,7 +7966,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:58</t>
+          <t>2026-03-11 17:37:40</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
@@ -8019,7 +8019,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:58</t>
+          <t>2026-03-11 17:37:40</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
@@ -8072,7 +8072,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:58</t>
+          <t>2026-03-11 17:37:40</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
@@ -8125,7 +8125,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:58</t>
+          <t>2026-03-11 17:37:40</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
@@ -8178,7 +8178,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:58</t>
+          <t>2026-03-11 17:37:40</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
@@ -8231,7 +8231,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:59</t>
+          <t>2026-03-11 17:37:41</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
@@ -8284,7 +8284,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:59</t>
+          <t>2026-03-11 17:37:41</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
@@ -8337,7 +8337,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:59</t>
+          <t>2026-03-11 17:37:41</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
@@ -8390,7 +8390,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:59</t>
+          <t>2026-03-11 17:37:41</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
@@ -8443,7 +8443,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:59</t>
+          <t>2026-03-11 17:37:41</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
@@ -8496,7 +8496,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:59</t>
+          <t>2026-03-11 17:37:41</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
@@ -8549,7 +8549,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:59</t>
+          <t>2026-03-11 17:37:41</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
@@ -8602,7 +8602,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:59</t>
+          <t>2026-03-11 17:37:41</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
@@ -8655,7 +8655,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:59</t>
+          <t>2026-03-11 17:37:41</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -8708,7 +8708,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:59</t>
+          <t>2026-03-11 17:37:41</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -8761,7 +8761,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>2026-03-11 16:55:59</t>
+          <t>2026-03-11 17:37:42</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:00</t>
+          <t>2026-03-11 17:37:42</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -8867,7 +8867,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:00</t>
+          <t>2026-03-11 17:37:42</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -8920,7 +8920,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:00</t>
+          <t>2026-03-11 17:37:42</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -8973,7 +8973,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:00</t>
+          <t>2026-03-11 17:37:42</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -9026,7 +9026,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:00</t>
+          <t>2026-03-11 17:37:42</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
@@ -9079,7 +9079,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:00</t>
+          <t>2026-03-11 17:37:42</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
@@ -9132,7 +9132,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:00</t>
+          <t>2026-03-11 17:37:42</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -9185,7 +9185,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:00</t>
+          <t>2026-03-11 17:37:42</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
@@ -9195,7 +9195,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>Reg 0x8A: OUT=0x000A, CE=0, STATUS=0 (OK)</t>
+          <t>Reg 0x8A: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -9238,7 +9238,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:00</t>
+          <t>2026-03-11 17:37:42</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>Reg 0x8B: OUT=0x0000, CE=0, STATUS=0 (OK)</t>
+          <t>Reg 0x8B: OUT=0x000A, CE=0, STATUS=0 (OK)</t>
         </is>
       </c>
     </row>
@@ -9291,7 +9291,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:00</t>
+          <t>2026-03-11 17:37:42</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
@@ -9344,7 +9344,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:01</t>
+          <t>2026-03-11 17:37:43</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
@@ -9397,7 +9397,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:01</t>
+          <t>2026-03-11 17:37:43</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
@@ -9450,7 +9450,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:01</t>
+          <t>2026-03-11 17:37:43</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
@@ -9503,7 +9503,7 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:01</t>
+          <t>2026-03-11 17:37:43</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
@@ -9556,7 +9556,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:01</t>
+          <t>2026-03-11 17:37:43</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
@@ -9609,7 +9609,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:01</t>
+          <t>2026-03-11 17:37:43</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
@@ -9662,7 +9662,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:01</t>
+          <t>2026-03-11 17:37:43</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
@@ -9715,7 +9715,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:01</t>
+          <t>2026-03-11 17:37:43</t>
         </is>
       </c>
       <c r="J150" t="inlineStr">
@@ -9768,7 +9768,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:01</t>
+          <t>2026-03-11 17:37:43</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
@@ -9821,7 +9821,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:01</t>
+          <t>2026-03-11 17:37:43</t>
         </is>
       </c>
       <c r="J152" t="inlineStr">
@@ -9874,7 +9874,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:02</t>
+          <t>2026-03-11 17:37:43</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
@@ -9927,7 +9927,7 @@
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:02</t>
+          <t>2026-03-11 17:37:44</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
@@ -9980,7 +9980,7 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:02</t>
+          <t>2026-03-11 17:37:44</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
@@ -10033,7 +10033,7 @@
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:02</t>
+          <t>2026-03-11 17:37:44</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
@@ -10086,7 +10086,7 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:02</t>
+          <t>2026-03-11 17:37:44</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
@@ -10139,7 +10139,7 @@
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:02</t>
+          <t>2026-03-11 17:37:44</t>
         </is>
       </c>
       <c r="J158" t="inlineStr">
@@ -10192,7 +10192,7 @@
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:02</t>
+          <t>2026-03-11 17:37:44</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
@@ -10245,7 +10245,7 @@
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:02</t>
+          <t>2026-03-11 17:37:44</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
@@ -10298,7 +10298,7 @@
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:02</t>
+          <t>2026-03-11 17:37:44</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
@@ -10351,7 +10351,7 @@
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:02</t>
+          <t>2026-03-11 17:37:44</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
@@ -10404,7 +10404,7 @@
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:02</t>
+          <t>2026-03-11 17:37:44</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
@@ -10457,7 +10457,7 @@
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:03</t>
+          <t>2026-03-11 17:37:45</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
@@ -10510,7 +10510,7 @@
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:03</t>
+          <t>2026-03-11 17:37:45</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
@@ -10563,7 +10563,7 @@
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:03</t>
+          <t>2026-03-11 17:37:45</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
@@ -10616,7 +10616,7 @@
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:03</t>
+          <t>2026-03-11 17:37:45</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
@@ -10669,7 +10669,7 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:03</t>
+          <t>2026-03-11 17:37:45</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
@@ -10722,7 +10722,7 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:03</t>
+          <t>2026-03-11 17:37:45</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
@@ -10775,7 +10775,7 @@
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:03</t>
+          <t>2026-03-11 17:37:45</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
@@ -10828,7 +10828,7 @@
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:03</t>
+          <t>2026-03-11 17:37:45</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
@@ -10881,7 +10881,7 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:03</t>
+          <t>2026-03-11 17:37:45</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
@@ -10934,7 +10934,7 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:03</t>
+          <t>2026-03-11 17:37:45</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
@@ -10987,7 +10987,7 @@
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:03</t>
+          <t>2026-03-11 17:37:45</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
@@ -11040,7 +11040,7 @@
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:04</t>
+          <t>2026-03-11 17:37:46</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
@@ -11093,7 +11093,7 @@
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:04</t>
+          <t>2026-03-11 17:37:46</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
@@ -11146,7 +11146,7 @@
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:04</t>
+          <t>2026-03-11 17:37:46</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
@@ -11199,7 +11199,7 @@
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:04</t>
+          <t>2026-03-11 17:37:46</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
@@ -11252,7 +11252,7 @@
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:04</t>
+          <t>2026-03-11 17:37:46</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
@@ -11305,7 +11305,7 @@
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:04</t>
+          <t>2026-03-11 17:37:46</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
@@ -11358,7 +11358,7 @@
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:04</t>
+          <t>2026-03-11 17:37:46</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
@@ -11411,7 +11411,7 @@
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:04</t>
+          <t>2026-03-11 17:37:46</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
@@ -11464,7 +11464,7 @@
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:04</t>
+          <t>2026-03-11 17:37:46</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
@@ -11517,7 +11517,7 @@
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:04</t>
+          <t>2026-03-11 17:37:46</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
@@ -11570,7 +11570,7 @@
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:05</t>
+          <t>2026-03-11 17:37:46</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
@@ -11623,7 +11623,7 @@
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:05</t>
+          <t>2026-03-11 17:37:47</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
@@ -11676,7 +11676,7 @@
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:05</t>
+          <t>2026-03-11 17:37:47</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
@@ -11729,7 +11729,7 @@
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:05</t>
+          <t>2026-03-11 17:37:47</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
@@ -11782,7 +11782,7 @@
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:05</t>
+          <t>2026-03-11 17:37:47</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
@@ -11835,7 +11835,7 @@
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:05</t>
+          <t>2026-03-11 17:37:47</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:05</t>
+          <t>2026-03-11 17:37:47</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
@@ -11941,7 +11941,7 @@
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:05</t>
+          <t>2026-03-11 17:37:47</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
@@ -11994,7 +11994,7 @@
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:05</t>
+          <t>2026-03-11 17:37:47</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
@@ -12047,7 +12047,7 @@
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:05</t>
+          <t>2026-03-11 17:37:47</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
@@ -12100,7 +12100,7 @@
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:05</t>
+          <t>2026-03-11 17:37:48</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
@@ -12153,7 +12153,7 @@
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:06</t>
+          <t>2026-03-11 17:37:48</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
@@ -12206,7 +12206,7 @@
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:06</t>
+          <t>2026-03-11 17:37:48</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
@@ -12259,7 +12259,7 @@
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:06</t>
+          <t>2026-03-11 17:37:48</t>
         </is>
       </c>
       <c r="J198" t="inlineStr">
@@ -12312,7 +12312,7 @@
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:06</t>
+          <t>2026-03-11 17:37:48</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
@@ -12365,7 +12365,7 @@
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:06</t>
+          <t>2026-03-11 17:37:48</t>
         </is>
       </c>
       <c r="J200" t="inlineStr">
@@ -12418,7 +12418,7 @@
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:06</t>
+          <t>2026-03-11 17:37:48</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
@@ -12471,7 +12471,7 @@
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:06</t>
+          <t>2026-03-11 17:37:48</t>
         </is>
       </c>
       <c r="J202" t="inlineStr">
@@ -12524,7 +12524,7 @@
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:06</t>
+          <t>2026-03-11 17:37:48</t>
         </is>
       </c>
       <c r="J203" t="inlineStr">
@@ -12577,7 +12577,7 @@
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:06</t>
+          <t>2026-03-11 17:37:48</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
@@ -12630,7 +12630,7 @@
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:06</t>
+          <t>2026-03-11 17:37:48</t>
         </is>
       </c>
       <c r="J205" t="inlineStr">
@@ -12683,7 +12683,7 @@
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:07</t>
+          <t>2026-03-11 17:37:49</t>
         </is>
       </c>
       <c r="J206" t="inlineStr">
@@ -12736,7 +12736,7 @@
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:07</t>
+          <t>2026-03-11 17:37:49</t>
         </is>
       </c>
       <c r="J207" t="inlineStr">
@@ -12789,7 +12789,7 @@
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:07</t>
+          <t>2026-03-11 17:37:49</t>
         </is>
       </c>
       <c r="J208" t="inlineStr">
@@ -12842,7 +12842,7 @@
       </c>
       <c r="I209" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:07</t>
+          <t>2026-03-11 17:37:49</t>
         </is>
       </c>
       <c r="J209" t="inlineStr">
@@ -12895,7 +12895,7 @@
       </c>
       <c r="I210" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:07</t>
+          <t>2026-03-11 17:37:49</t>
         </is>
       </c>
       <c r="J210" t="inlineStr">
@@ -12948,7 +12948,7 @@
       </c>
       <c r="I211" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:07</t>
+          <t>2026-03-11 17:37:49</t>
         </is>
       </c>
       <c r="J211" t="inlineStr">
@@ -13001,7 +13001,7 @@
       </c>
       <c r="I212" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:07</t>
+          <t>2026-03-11 17:37:49</t>
         </is>
       </c>
       <c r="J212" t="inlineStr">
@@ -13054,7 +13054,7 @@
       </c>
       <c r="I213" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:07</t>
+          <t>2026-03-11 17:37:49</t>
         </is>
       </c>
       <c r="J213" t="inlineStr">
@@ -13107,7 +13107,7 @@
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:07</t>
+          <t>2026-03-11 17:37:49</t>
         </is>
       </c>
       <c r="J214" t="inlineStr">
@@ -13160,7 +13160,7 @@
       </c>
       <c r="I215" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:07</t>
+          <t>2026-03-11 17:37:49</t>
         </is>
       </c>
       <c r="J215" t="inlineStr">
@@ -13213,7 +13213,7 @@
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:08</t>
+          <t>2026-03-11 17:37:49</t>
         </is>
       </c>
       <c r="J216" t="inlineStr">
@@ -13266,7 +13266,7 @@
       </c>
       <c r="I217" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:08</t>
+          <t>2026-03-11 17:37:50</t>
         </is>
       </c>
       <c r="J217" t="inlineStr">
@@ -13319,7 +13319,7 @@
       </c>
       <c r="I218" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:08</t>
+          <t>2026-03-11 17:37:50</t>
         </is>
       </c>
       <c r="J218" t="inlineStr">
@@ -13372,7 +13372,7 @@
       </c>
       <c r="I219" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:08</t>
+          <t>2026-03-11 17:37:50</t>
         </is>
       </c>
       <c r="J219" t="inlineStr">
@@ -13425,7 +13425,7 @@
       </c>
       <c r="I220" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:08</t>
+          <t>2026-03-11 17:37:50</t>
         </is>
       </c>
       <c r="J220" t="inlineStr">
@@ -13478,7 +13478,7 @@
       </c>
       <c r="I221" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:08</t>
+          <t>2026-03-11 17:37:50</t>
         </is>
       </c>
       <c r="J221" t="inlineStr">
@@ -13531,7 +13531,7 @@
       </c>
       <c r="I222" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:08</t>
+          <t>2026-03-11 17:37:50</t>
         </is>
       </c>
       <c r="J222" t="inlineStr">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="I223" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:08</t>
+          <t>2026-03-11 17:37:50</t>
         </is>
       </c>
       <c r="J223" t="inlineStr">
@@ -13637,7 +13637,7 @@
       </c>
       <c r="I224" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:08</t>
+          <t>2026-03-11 17:37:50</t>
         </is>
       </c>
       <c r="J224" t="inlineStr">
@@ -13690,7 +13690,7 @@
       </c>
       <c r="I225" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:08</t>
+          <t>2026-03-11 17:37:50</t>
         </is>
       </c>
       <c r="J225" t="inlineStr">
@@ -13743,7 +13743,7 @@
       </c>
       <c r="I226" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:08</t>
+          <t>2026-03-11 17:37:50</t>
         </is>
       </c>
       <c r="J226" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="I227" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:09</t>
+          <t>2026-03-11 17:37:51</t>
         </is>
       </c>
       <c r="J227" t="inlineStr">
@@ -13849,7 +13849,7 @@
       </c>
       <c r="I228" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:09</t>
+          <t>2026-03-11 17:37:51</t>
         </is>
       </c>
       <c r="J228" t="inlineStr">
@@ -13902,7 +13902,7 @@
       </c>
       <c r="I229" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:09</t>
+          <t>2026-03-11 17:37:51</t>
         </is>
       </c>
       <c r="J229" t="inlineStr">
@@ -13955,7 +13955,7 @@
       </c>
       <c r="I230" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:09</t>
+          <t>2026-03-11 17:37:51</t>
         </is>
       </c>
       <c r="J230" t="inlineStr">
@@ -14008,7 +14008,7 @@
       </c>
       <c r="I231" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:09</t>
+          <t>2026-03-11 17:37:51</t>
         </is>
       </c>
       <c r="J231" t="inlineStr">
@@ -14061,7 +14061,7 @@
       </c>
       <c r="I232" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:09</t>
+          <t>2026-03-11 17:37:51</t>
         </is>
       </c>
       <c r="J232" t="inlineStr">
@@ -14114,7 +14114,7 @@
       </c>
       <c r="I233" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:09</t>
+          <t>2026-03-11 17:37:51</t>
         </is>
       </c>
       <c r="J233" t="inlineStr">
@@ -14167,7 +14167,7 @@
       </c>
       <c r="I234" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:09</t>
+          <t>2026-03-11 17:37:51</t>
         </is>
       </c>
       <c r="J234" t="inlineStr">
@@ -14220,7 +14220,7 @@
       </c>
       <c r="I235" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:09</t>
+          <t>2026-03-11 17:37:51</t>
         </is>
       </c>
       <c r="J235" t="inlineStr">
@@ -14273,7 +14273,7 @@
       </c>
       <c r="I236" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:09</t>
+          <t>2026-03-11 17:37:51</t>
         </is>
       </c>
       <c r="J236" t="inlineStr">
@@ -14326,7 +14326,7 @@
       </c>
       <c r="I237" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:10</t>
+          <t>2026-03-11 17:37:51</t>
         </is>
       </c>
       <c r="J237" t="inlineStr">
@@ -14379,7 +14379,7 @@
       </c>
       <c r="I238" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:10</t>
+          <t>2026-03-11 17:37:52</t>
         </is>
       </c>
       <c r="J238" t="inlineStr">
@@ -14432,7 +14432,7 @@
       </c>
       <c r="I239" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:10</t>
+          <t>2026-03-11 17:37:52</t>
         </is>
       </c>
       <c r="J239" t="inlineStr">
@@ -14485,7 +14485,7 @@
       </c>
       <c r="I240" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:10</t>
+          <t>2026-03-11 17:37:52</t>
         </is>
       </c>
       <c r="J240" t="inlineStr">
@@ -14538,7 +14538,7 @@
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:10</t>
+          <t>2026-03-11 17:37:52</t>
         </is>
       </c>
       <c r="J241" t="inlineStr">
@@ -14591,7 +14591,7 @@
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:10</t>
+          <t>2026-03-11 17:37:52</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
@@ -14644,7 +14644,7 @@
       </c>
       <c r="I243" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:10</t>
+          <t>2026-03-11 17:37:52</t>
         </is>
       </c>
       <c r="J243" t="inlineStr">
@@ -14697,7 +14697,7 @@
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:10</t>
+          <t>2026-03-11 17:37:52</t>
         </is>
       </c>
       <c r="J244" t="inlineStr">
@@ -14750,7 +14750,7 @@
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:10</t>
+          <t>2026-03-11 17:37:52</t>
         </is>
       </c>
       <c r="J245" t="inlineStr">
@@ -14803,7 +14803,7 @@
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:10</t>
+          <t>2026-03-11 17:37:52</t>
         </is>
       </c>
       <c r="J246" t="inlineStr">
@@ -14856,7 +14856,7 @@
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:10</t>
+          <t>2026-03-11 17:37:52</t>
         </is>
       </c>
       <c r="J247" t="inlineStr">
@@ -14909,7 +14909,7 @@
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:11</t>
+          <t>2026-03-11 17:37:53</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
@@ -14962,7 +14962,7 @@
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:11</t>
+          <t>2026-03-11 17:37:53</t>
         </is>
       </c>
       <c r="J249" t="inlineStr">
@@ -15015,7 +15015,7 @@
       </c>
       <c r="I250" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:11</t>
+          <t>2026-03-11 17:37:53</t>
         </is>
       </c>
       <c r="J250" t="inlineStr">
@@ -15068,7 +15068,7 @@
       </c>
       <c r="I251" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:11</t>
+          <t>2026-03-11 17:37:53</t>
         </is>
       </c>
       <c r="J251" t="inlineStr">
@@ -15121,7 +15121,7 @@
       </c>
       <c r="I252" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:11</t>
+          <t>2026-03-11 17:37:53</t>
         </is>
       </c>
       <c r="J252" t="inlineStr">
@@ -15174,7 +15174,7 @@
       </c>
       <c r="I253" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:11</t>
+          <t>2026-03-11 17:37:53</t>
         </is>
       </c>
       <c r="J253" t="inlineStr">
@@ -15227,7 +15227,7 @@
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:11</t>
+          <t>2026-03-11 17:37:53</t>
         </is>
       </c>
       <c r="J254" t="inlineStr">
@@ -15280,7 +15280,7 @@
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:11</t>
+          <t>2026-03-11 17:37:53</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
@@ -15333,7 +15333,7 @@
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:11</t>
+          <t>2026-03-11 17:37:53</t>
         </is>
       </c>
       <c r="J256" t="inlineStr">
@@ -15386,7 +15386,7 @@
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:11</t>
+          <t>2026-03-11 17:37:53</t>
         </is>
       </c>
       <c r="J257" t="inlineStr">
@@ -15525,7 +15525,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:12</t>
+          <t>2026-03-11 17:37:54</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -15559,7 +15559,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:13</t>
+          <t>2026-03-11 17:37:55</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -15593,7 +15593,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:14</t>
+          <t>2026-03-11 17:37:56</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -15627,7 +15627,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:15</t>
+          <t>2026-03-11 17:37:57</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -15661,7 +15661,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:16</t>
+          <t>2026-03-11 17:37:58</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -15720,12 +15720,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ERROR: name 'write_tuners' is not defined</t>
+          <t>Wrote phase=12.12,ring1=9.99,ring2=5.55 | Read phase=12.120,ring1=9.990,ring2=5.550</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -15735,7 +15735,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:18</t>
+          <t>2026-03-11 17:38:01</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -15752,12 +15752,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ERROR: name 'write_soa' is not defined</t>
+          <t>Wrote soa=1.23 | Read soa=1.23</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -15767,7 +15767,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:18</t>
+          <t>2026-03-11 17:38:01</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -15784,12 +15784,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ERROR: name 'write_bias' is not defined</t>
+          <t>Wrote bias=123 | Read bias=123</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -15799,7 +15799,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:18</t>
+          <t>2026-03-11 17:38:01</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -15816,12 +15816,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ERROR: name 'write_tec' is not defined</t>
+          <t>Wrote tec=-45 | Read tec=-45</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -15831,7 +15831,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:18</t>
+          <t>2026-03-11 17:38:02</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -16001,7 +16001,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:19</t>
+          <t>2026-03-11 17:38:02</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -16038,7 +16038,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:19</t>
+          <t>2026-03-11 17:38:03</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -16075,7 +16075,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:20</t>
+          <t>2026-03-11 17:38:03</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -16112,7 +16112,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:20</t>
+          <t>2026-03-11 17:38:03</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -16149,7 +16149,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:20</t>
+          <t>2026-03-11 17:38:04</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -16186,7 +16186,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:20</t>
+          <t>2026-03-11 17:38:04</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -16223,7 +16223,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-03-11 16:56:21</t>
+          <t>2026-03-11 17:38:04</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">

</xml_diff>